<commit_message>
file save decimal precision fix
</commit_message>
<xml_diff>
--- a/Docs/NI USB 6526 IO Device.xlsx
+++ b/Docs/NI USB 6526 IO Device.xlsx
@@ -5,16 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nanometa\Documents\LabVIEW Data\TCSPC\Diagrams manuals notes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nanometa\Documents\TCSPC_Git_Repo\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A9966CF-1C40-4662-BED5-13C826E925FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{159A073A-C45F-4597-9CC8-B3B3E5AE79CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="2" xr2:uid="{3516360F-1565-4B63-B275-BFEAF3C8E0D9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="1" xr2:uid="{3516360F-1565-4B63-B275-BFEAF3C8E0D9}"/>
   </bookViews>
   <sheets>
     <sheet name="USB-6525" sheetId="1" r:id="rId1"/>
-    <sheet name="USB-6351" sheetId="2" r:id="rId2"/>
+    <sheet name="USB-6341" sheetId="2" r:id="rId2"/>
     <sheet name="Delay Line Configuration" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -463,14 +463,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -480,15 +484,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1408,7 +1403,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:H8 J2:J4 J7">
+  <conditionalFormatting sqref="J2:J4 E2:H8 J7">
     <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="T">
       <formula>NOT(ISERROR(SEARCH("T",E2)))</formula>
     </cfRule>
@@ -1428,7 +1423,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.85546875" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" customWidth="1"/>
     <col min="3" max="3" width="26.7109375" customWidth="1"/>
     <col min="4" max="4" width="21.7109375" customWidth="1"/>
   </cols>
@@ -1521,28 +1516,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="9"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="13"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1550,51 +1545,50 @@
       <c r="A3" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3">
         <v>498</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2">
+      <c r="D3">
         <v>498</v>
       </c>
-      <c r="E3" s="3"/>
+      <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="4">
         <v>1440</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5">
+      <c r="C4" s="4"/>
+      <c r="D4" s="4">
         <v>1060</v>
       </c>
-      <c r="E4" s="6"/>
+      <c r="E4" s="5"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="9"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="13"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" t="s">
         <v>73</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" t="s">
         <v>74</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" s="2" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1602,39 +1596,38 @@
       <c r="A8" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" t="s">
         <v>90</v>
       </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2" t="s">
+      <c r="D8" t="s">
         <v>90</v>
       </c>
-      <c r="E8" s="3"/>
+      <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="4">
         <v>1440</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5">
+      <c r="C9" s="4"/>
+      <c r="D9" s="4">
         <v>1060</v>
       </c>
-      <c r="E9" s="6"/>
+      <c r="E9" s="5"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" t="s">
         <v>84</v>
       </c>
     </row>
@@ -1642,10 +1635,10 @@
       <c r="A12" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" t="s">
         <v>86</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="9" t="s">
         <v>88</v>
       </c>
     </row>
@@ -1653,21 +1646,21 @@
       <c r="A13" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="B13" s="15" t="s">
+      <c r="B13" t="s">
         <v>85</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="9" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="10" t="s">
         <v>89</v>
       </c>
     </row>

</xml_diff>